<commit_message>
Plan: 35 of 35 automatable cases done (CCCT-2671)
Stamps the six cases closed today - TC-BRD-004, TC-CAL-006, TC-KWD-004/005,
TC-CHN-005/006 - and TC-CHN-003 now that a reserved account exists for it.

TC-CHN-005 needed no new code: the guard it describes already runs 16 times
across 6 flows before every send.

The Coverage Summary is formulas over these sheets, so it recomputes itself.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Messaging_Workflow_Automation_Test_Plan.xlsx
+++ b/Messaging_Workflow_Automation_Test_Plan.xlsx
@@ -2665,13 +2665,17 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>M3 messaging_empty_state.yaml</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr"/>
+          <t>test_messaging_hybrid::test_channel_list_shows_empty_state + messaging_empty_state.yaml</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Legacy verify_channel_list() accepts empty OR populated, so it pins neither state. The flow is written and passed once (staging, build e008c256) but is NOT currently reproducible: it needs an account that has never been in ANY channel on ANY domain, and no such account is reserved. Message Automation User qualified until it gained a channel; Deb Test 8/12 already carries channels from other domains (connetqa-prod, connectqa). This is a fragile resource by nature - any bulk consent request on a domain a worker belongs to populates it. Needs a dedicated never-enrolled PersonalID number, or the flow changed to sign UP a fresh account per run, which by definition has no channels.</t>
+          <t>The flow existed and was registered but nothing ran it - the only reference in the suite was a comment - so this needed a test wrapper as well as an account. Runs as MAESTRO_MESSAGING_EMPTY_STATE, a reserved pair (prod 4376447 / staging 4376448) that must never be invited to a channel or an opportunity: a channel cannot be undone, so one consent request retires this case permanently. Verified on prod, build 842ed35d. A failure here most likely means the account picked up a channel rather than that the empty state is broken.</t>
         </is>
       </c>
     </row>
@@ -2750,10 +2754,14 @@
           <t>Shared precondition step (all flows)</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr"/>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Not a user-facing case - a guard. Without it, a key-sync failure and a genuine delivery failure look identical, and we would chase a phantom product bug. MessagingChannelsKeySyncWorker backfills keys for consented keyless channels.</t>
+          <t>Already covered, no separate flow needed: the sequence this case describes - open the channel, type into etMessage, assert imgSendMessage appears - occurs 16 times across 6 messaging flows, before every send. That is exactly the guard the case asks for.</t>
         </is>
       </c>
     </row>
@@ -2786,13 +2794,17 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>M2 messaging_subscription.yaml</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr"/>
+          <t>test_messaging_hybrid::test_subscribed_channels_sort_before_unsubscribed + messaging_subscription.yaml</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>ChannelAdapter.setChannels. Cheap to assert once TC-SUB-001 has produced an unsubscribed channel in the same session.</t>
+          <t>Needs no hand-prepared account. The worker holds several channels and all are subscribed, so the flow unsubscribes a spare itself and restores it, and repairs the state if a previous run died mid-way. The spare is never the channel the delivery tests send into. It asserts position BEFORE and after: the first spare tried sorted last, so unsubscribing it moved nothing and the case would have passed without observing a sort at all. The within-subscribed order is not stable day to day, so that starting-order assert is what keeps a changed order loud rather than quiet.</t>
         </is>
       </c>
     </row>
@@ -3081,13 +3093,17 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>W2 test_messaging_broadcasts</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr"/>
+          <t>test_messaging_hybrid::test_broadcast_connect_survey_is_answerable + messaging_survey.yaml</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>GAP vs legacy. The manual outcome requires 'Form should get submit and able to verify it on the submit history'; legacy never checks HQ received anything, so a survey that renders but never submits would pass today.</t>
+          <t>Asserted in the same test that answers the survey rather than as a separate run: one device build proves both. Submissions are attributed to the Connect user id, not the PersonalID mobile worker - searching by mobile worker returns nothing while the row is sitting there, which is why this looked blocked. The search is bounded by a timestamp taken before the send, so a previous run's submission cannot satisfy it.</t>
         </is>
       </c>
     </row>
@@ -3416,13 +3432,17 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>W1 test_messaging_conditional_alerts</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr"/>
+          <t>test_messaging_hybrid::test_conditional_alert_survey_is_answerable + messaging_conditional_alert_survey.yaml</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>GAP vs legacy - same as TC-BRD-004.</t>
+          <t>Same submit-history check as TC-BRD-004. Matched on the full survey_form breadcrumb rather than 'Registration Form': this flow also submits a Delivery App Registration Form to fire the alert, and a loose match would assert on that one instead.</t>
         </is>
       </c>
     </row>
@@ -3701,13 +3721,17 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>W4 test_messaging_keywords</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr"/>
+          <t>test_messaging_hybrid::test_keyword_returns_a_survey_that_is_answerable + messaging_keyword_survey.yaml</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Manual 'Connect message6'.</t>
+          <t>Was never actually written - the hybrid module's docstring claimed it, but only TC-KWD-002 existed. The flow is the send half of messaging_keyword.yaml followed by the answering half of messaging_survey.yaml. Worth its own case: TC-KWD-002's reply is a single canned message, whereas each question here arrives only after the previous is answered.</t>
         </is>
       </c>
     </row>
@@ -3739,13 +3763,17 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>W4 test_messaging_keywords</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr"/>
+          <t>test_messaging_hybrid::test_keyword_returns_a_survey_that_is_answerable + messaging_keyword_survey.yaml</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Explicit in the manual outcome for 'Connect message6'.</t>
+          <t>Same submit-history check as TC-BRD-004, asserted in the same run as TC-KWD-004.</t>
         </is>
       </c>
     </row>

</xml_diff>